<commit_message>
fix(liquidacao): placares manuais restaurados e conferidos pela rotina noturna
Os placares de 29-30/08 da mestre e das planilhas diárias 03-09/09 foram
preenchidos manualmente pelo Thiago — não por pipeline, como eu havia assumido.
O achado se mantém (23 de 42 divergem de duas bases independentes que concordam
entre si; 5 falsos GREEN), mas a causa provável é digitação ou placar consultado
antes do fim, e a redação no worklog e na memória foi corrigida.

Desfeito: eu tinha zerado para PENDENTE 60 linhas manuais de 03-09/09.
Restauradas como Fonte_Placar=manual, em liability/5%.

liquidar_resultados_noite: linhas manuais deixam de ser ignoradas — quando a
base cobre o jogo, confere; se divergir, a base vence, o manual fica em
*_Original e a divergência é listada no fechamento. Sem base ainda, o manual
continua valendo.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/metodos_aprovados/Sinais_Metodos_Aprovados_2026-09-03.xlsx
+++ b/metodos_aprovados/Sinais_Metodos_Aprovados_2026-09-03.xlsx
@@ -724,15 +724,17 @@
       </c>
       <c r="N3" t="inlineStr">
         <is>
-          <t>?</t>
+          <t>0x2</t>
         </is>
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr"/>
+          <t>GREEN</t>
+        </is>
+      </c>
+      <c r="P3" t="n">
+        <v>1</v>
+      </c>
       <c r="Q3" t="n">
         <v>0.95</v>
       </c>
@@ -741,11 +743,25 @@
           <t>GREEN</t>
         </is>
       </c>
-      <c r="S3" t="inlineStr"/>
-      <c r="T3" t="inlineStr"/>
-      <c r="U3" t="inlineStr"/>
-      <c r="V3" t="inlineStr"/>
-      <c r="W3" t="inlineStr"/>
+      <c r="S3" t="n">
+        <v>0.16964</v>
+      </c>
+      <c r="T3" t="n">
+        <v>16.96</v>
+      </c>
+      <c r="U3" t="inlineStr">
+        <is>
+          <t>manual</t>
+        </is>
+      </c>
+      <c r="V3" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>LIABILITY=1u;comissao=5%</t>
+        </is>
+      </c>
       <c r="X3" t="inlineStr">
         <is>
           <t>0x2</t>

</xml_diff>

<commit_message>
revert(liquidacao): tudo de volta ao estado manual do Thiago; 23:30 só avisa divergência
Decisão do usuário (opção A). Mestre, planilhas diárias 03-09/09 e
automacao_diaria_aprovados.py restaurados dos backups .bak_20260911.
Scripts que escreviam nas planilhas arquivados em _arquivados_11set/.
Novo conferir_placares_manuais.py só lista divergências planilha x base no
Telegram, sem alterar nada. Auditoria fica como registro.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/metodos_aprovados/Sinais_Metodos_Aprovados_2026-09-03.xlsx
+++ b/metodos_aprovados/Sinais_Metodos_Aprovados_2026-09-03.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y3"/>
+  <dimension ref="A1:T3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -529,31 +529,6 @@
           <t>PnL_R$</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>Fonte_Placar</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>PnL_stake_u</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>Convencao_PnL</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>Placar_Original</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>Resultado_Original</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -635,33 +610,10 @@
         </is>
       </c>
       <c r="S2" t="n">
-        <v>0.19388</v>
+        <v>0.95</v>
       </c>
       <c r="T2" t="n">
         <v>19.39</v>
-      </c>
-      <c r="U2" t="inlineStr">
-        <is>
-          <t>betfair:fuzzy0.96</t>
-        </is>
-      </c>
-      <c r="V2" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>LIABILITY=1u;comissao=5%</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>4x0</t>
-        </is>
-      </c>
-      <c r="Y2" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
       </c>
     </row>
     <row r="3">
@@ -744,33 +696,10 @@
         </is>
       </c>
       <c r="S3" t="n">
-        <v>0.16964</v>
+        <v>0.95</v>
       </c>
       <c r="T3" t="n">
-        <v>16.96</v>
-      </c>
-      <c r="U3" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-      <c r="V3" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>LIABILITY=1u;comissao=5%</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>0x2</t>
-        </is>
-      </c>
-      <c r="Y3" t="inlineStr">
-        <is>
-          <t>GREEN</t>
-        </is>
+        <v>16.97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>